<commit_message>
Implement ETL data cleaning pipeline and processed datasets
</commit_message>
<xml_diff>
--- a/data/raw/issue_log.xlsx
+++ b/data/raw/issue_log.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2" conformance="strict">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2" conformance="strict">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
   <workbookPr dateCompatibility="0" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="7514" uniqueCount="1305">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7514" uniqueCount="1305">
   <si>
     <t>Issue ID</t>
   </si>
@@ -3945,7 +3945,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -4801,7 +4801,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B21CECF3-9B51-B346-A23A-23638F56C505}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B21CECF3-9B51-B346-A23A-23638F56C505}">
   <dimension ref="A1:N751"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>